<commit_message>
fix bug not fill purchase link in DNTU
</commit_message>
<xml_diff>
--- a/SourceCode/EV_ERP/EV_ERP/wwwroot/templates/DNTU-template.xlsx
+++ b/SourceCode/EV_ERP/EV_ERP/wwwroot/templates/DNTU-template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Dev\EV_ERP\SourceCode\EV_ERP\EV_ERP\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20C3775B-F7A3-4CB7-9ABB-76F81E77466D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A33C975C-5158-4D50-8174-FF317AD2C77B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ĐNTU" sheetId="1" r:id="rId1"/>
@@ -217,7 +217,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="82" uniqueCount="64">
   <si>
     <t>CÔNG TY CỔ PHẦN TƯ VẤN THIẾT BỊ EASTERN VISION
 EASTERN VISION EQUIPMENT CONSULTANCY .,JSC</t>
@@ -496,9 +496,6 @@
   </si>
   <si>
     <t>20.04.2026</t>
-  </si>
-  <si>
-    <t>https://shopee.vn/20-N%C3%BAt-%C4%91%E1%BB%87m-cao-su-3M-SJ5312-(N%C3%BAt-d%E1%BA%B9t)-V%C3%A0-30-N%C3%BAt-3MSJ5302-(N%C3%BAt-V%C3%B2m-Nh%E1%BB%8F)-i.50663522.7926817811?sp_atk=12653609-96c4-49c5-ad3a-5eb6b2bceb18&amp;xptdk=12653609-96c4-49c5-ad3a-5eb6b2bceb18</t>
   </si>
   <si>
     <t>Ngày: 03/04/2026</t>
@@ -1349,6 +1346,72 @@
     <xf numFmtId="164" fontId="41" fillId="2" borderId="2" xfId="8" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="36" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="21" fillId="3" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="37" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="23" fillId="9" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="7" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="11" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="16" fillId="11" borderId="2" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="22" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="17" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="16" fillId="5" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="26" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="166" fontId="34" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1358,15 +1421,6 @@
     <xf numFmtId="166" fontId="23" fillId="8" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="28" fillId="13" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="28" fillId="13" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="24" fillId="7" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="165" fontId="19" fillId="14" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1405,63 +1459,6 @@
     </xf>
     <xf numFmtId="166" fontId="16" fillId="8" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="17" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="2" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="3" fontId="16" fillId="5" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="2" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="26" fillId="2" borderId="6" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="2" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="36" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="21" fillId="3" borderId="2" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="37" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="23" fillId="9" borderId="2" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="11" borderId="2" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="16" fillId="11" borderId="2" xfId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="22" fillId="6" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="9">
@@ -1843,75 +1840,75 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:V41"/>
-  <sheetFormatPr defaultColWidth="8.44140625" defaultRowHeight="46.2"/>
+  <sheetFormatPr defaultColWidth="8.42578125" defaultRowHeight="45.75"/>
   <cols>
-    <col min="1" max="1" width="12.88671875" style="6" customWidth="1"/>
-    <col min="2" max="2" width="26.6640625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="52.33203125" style="2" customWidth="1"/>
-    <col min="4" max="4" width="14.6640625" style="7" customWidth="1"/>
-    <col min="5" max="5" width="12.6640625" style="6" customWidth="1"/>
-    <col min="6" max="6" width="23.33203125" style="5" customWidth="1"/>
-    <col min="7" max="7" width="19.5546875" style="11" customWidth="1"/>
-    <col min="8" max="8" width="23.33203125" style="2" customWidth="1"/>
-    <col min="9" max="9" width="3.88671875" style="2" customWidth="1"/>
-    <col min="10" max="10" width="24.5546875" style="4" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" style="6" customWidth="1"/>
+    <col min="2" max="2" width="26.7109375" style="6" customWidth="1"/>
+    <col min="3" max="3" width="52.28515625" style="2" customWidth="1"/>
+    <col min="4" max="4" width="14.7109375" style="7" customWidth="1"/>
+    <col min="5" max="5" width="12.7109375" style="6" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" style="5" customWidth="1"/>
+    <col min="7" max="7" width="19.5703125" style="11" customWidth="1"/>
+    <col min="8" max="8" width="23.28515625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="3.85546875" style="2" customWidth="1"/>
+    <col min="10" max="10" width="24.5703125" style="4" customWidth="1"/>
     <col min="11" max="11" width="14" style="2" customWidth="1"/>
-    <col min="12" max="12" width="23.33203125" style="2" customWidth="1"/>
-    <col min="13" max="13" width="11.88671875" style="6" customWidth="1"/>
-    <col min="14" max="14" width="19.44140625" style="6" customWidth="1"/>
-    <col min="15" max="15" width="26.44140625" style="2" customWidth="1"/>
+    <col min="12" max="12" width="23.28515625" style="2" customWidth="1"/>
+    <col min="13" max="13" width="11.85546875" style="6" customWidth="1"/>
+    <col min="14" max="14" width="19.42578125" style="6" customWidth="1"/>
+    <col min="15" max="15" width="26.42578125" style="2" customWidth="1"/>
     <col min="16" max="16" width="15" style="6" customWidth="1"/>
-    <col min="17" max="18" width="21.88671875" style="4" customWidth="1"/>
-    <col min="19" max="19" width="30.88671875" style="3" customWidth="1"/>
+    <col min="17" max="18" width="21.85546875" style="4" customWidth="1"/>
+    <col min="19" max="19" width="30.85546875" style="3" customWidth="1"/>
     <col min="20" max="20" width="27" style="80" customWidth="1"/>
-    <col min="21" max="16384" width="8.44140625" style="2"/>
+    <col min="21" max="16384" width="8.42578125" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="98.7" customHeight="1">
+    <row r="1" spans="1:20" ht="98.65" customHeight="1">
       <c r="A1" s="1"/>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="E1" s="72"/>
       <c r="F1" s="14"/>
-      <c r="G1" s="155" t="s">
+      <c r="G1" s="124" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="155"/>
-      <c r="I1" s="155"/>
-      <c r="J1" s="155"/>
-      <c r="K1" s="155"/>
-      <c r="L1" s="155"/>
-      <c r="M1" s="155"/>
-      <c r="N1" s="155"/>
-      <c r="O1" s="155"/>
-      <c r="P1" s="155"/>
-      <c r="Q1" s="155"/>
-      <c r="R1" s="155"/>
-      <c r="S1" s="155"/>
-      <c r="T1" s="155"/>
-    </row>
-    <row r="2" spans="1:20" ht="55.95" customHeight="1">
+      <c r="H1" s="124"/>
+      <c r="I1" s="124"/>
+      <c r="J1" s="124"/>
+      <c r="K1" s="124"/>
+      <c r="L1" s="124"/>
+      <c r="M1" s="124"/>
+      <c r="N1" s="124"/>
+      <c r="O1" s="124"/>
+      <c r="P1" s="124"/>
+      <c r="Q1" s="124"/>
+      <c r="R1" s="124"/>
+      <c r="S1" s="124"/>
+      <c r="T1" s="124"/>
+    </row>
+    <row r="2" spans="1:20" ht="55.9" customHeight="1">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="E2" s="13"/>
       <c r="F2" s="12"/>
-      <c r="G2" s="157" t="s">
+      <c r="G2" s="126" t="s">
         <v>46</v>
       </c>
-      <c r="H2" s="157"/>
-      <c r="I2" s="157"/>
-      <c r="J2" s="157"/>
-      <c r="K2" s="157"/>
-      <c r="L2" s="157"/>
-      <c r="M2" s="157"/>
-      <c r="N2" s="157"/>
-      <c r="O2" s="157"/>
-      <c r="P2" s="157"/>
-      <c r="Q2" s="157"/>
-      <c r="R2" s="157"/>
-      <c r="S2" s="157"/>
-      <c r="T2" s="157"/>
+      <c r="H2" s="126"/>
+      <c r="I2" s="126"/>
+      <c r="J2" s="126"/>
+      <c r="K2" s="126"/>
+      <c r="L2" s="126"/>
+      <c r="M2" s="126"/>
+      <c r="N2" s="126"/>
+      <c r="O2" s="126"/>
+      <c r="P2" s="126"/>
+      <c r="Q2" s="126"/>
+      <c r="R2" s="126"/>
+      <c r="S2" s="126"/>
+      <c r="T2" s="126"/>
     </row>
     <row r="3" spans="1:20" ht="64.5" customHeight="1">
       <c r="A3" s="1"/>
@@ -1919,46 +1916,46 @@
       <c r="C3" s="1"/>
       <c r="E3" s="13"/>
       <c r="F3" s="12"/>
-      <c r="G3" s="157" t="s">
+      <c r="G3" s="126" t="s">
         <v>1</v>
       </c>
-      <c r="H3" s="157"/>
-      <c r="I3" s="157"/>
-      <c r="J3" s="157"/>
-      <c r="K3" s="157"/>
-      <c r="L3" s="157"/>
-      <c r="M3" s="157"/>
-      <c r="N3" s="157"/>
-      <c r="O3" s="157"/>
-      <c r="P3" s="157"/>
-      <c r="Q3" s="157"/>
-      <c r="R3" s="157"/>
-      <c r="S3" s="157"/>
-      <c r="T3" s="157"/>
+      <c r="H3" s="126"/>
+      <c r="I3" s="126"/>
+      <c r="J3" s="126"/>
+      <c r="K3" s="126"/>
+      <c r="L3" s="126"/>
+      <c r="M3" s="126"/>
+      <c r="N3" s="126"/>
+      <c r="O3" s="126"/>
+      <c r="P3" s="126"/>
+      <c r="Q3" s="126"/>
+      <c r="R3" s="126"/>
+      <c r="S3" s="126"/>
+      <c r="T3" s="126"/>
     </row>
     <row r="4" spans="1:20" ht="67.5" customHeight="1">
-      <c r="A4" s="156" t="s">
+      <c r="A4" s="125" t="s">
         <v>33</v>
       </c>
-      <c r="B4" s="156"/>
-      <c r="C4" s="156"/>
-      <c r="D4" s="156"/>
-      <c r="E4" s="156"/>
-      <c r="F4" s="156"/>
-      <c r="G4" s="156"/>
-      <c r="H4" s="156"/>
-      <c r="I4" s="156"/>
-      <c r="J4" s="156"/>
-      <c r="K4" s="156"/>
-      <c r="L4" s="156"/>
-      <c r="M4" s="156"/>
-      <c r="N4" s="156"/>
-      <c r="O4" s="156"/>
-      <c r="P4" s="156"/>
-      <c r="Q4" s="156"/>
-      <c r="R4" s="156"/>
-      <c r="S4" s="156"/>
-      <c r="T4" s="156"/>
+      <c r="B4" s="125"/>
+      <c r="C4" s="125"/>
+      <c r="D4" s="125"/>
+      <c r="E4" s="125"/>
+      <c r="F4" s="125"/>
+      <c r="G4" s="125"/>
+      <c r="H4" s="125"/>
+      <c r="I4" s="125"/>
+      <c r="J4" s="125"/>
+      <c r="K4" s="125"/>
+      <c r="L4" s="125"/>
+      <c r="M4" s="125"/>
+      <c r="N4" s="125"/>
+      <c r="O4" s="125"/>
+      <c r="P4" s="125"/>
+      <c r="Q4" s="125"/>
+      <c r="R4" s="125"/>
+      <c r="S4" s="125"/>
+      <c r="T4" s="125"/>
     </row>
     <row r="5" spans="1:20" s="4" customFormat="1">
       <c r="A5" s="15" t="s">
@@ -1967,19 +1964,19 @@
       <c r="B5" s="15"/>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
-      <c r="E5" s="161" t="s">
+      <c r="E5" s="133" t="s">
         <v>51</v>
       </c>
-      <c r="F5" s="161"/>
-      <c r="G5" s="161"/>
+      <c r="F5" s="133"/>
+      <c r="G5" s="133"/>
       <c r="H5" s="103"/>
       <c r="I5" s="49"/>
-      <c r="K5" s="145" t="s">
+      <c r="K5" s="136" t="s">
         <v>50</v>
       </c>
-      <c r="L5" s="145"/>
-      <c r="M5" s="145"/>
-      <c r="N5" s="145"/>
+      <c r="L5" s="136"/>
+      <c r="M5" s="136"/>
+      <c r="N5" s="136"/>
       <c r="O5" s="50"/>
       <c r="P5" s="88"/>
       <c r="Q5" s="18"/>
@@ -1993,7 +1990,7 @@
       </c>
       <c r="B6" s="51"/>
       <c r="C6" s="51" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D6" s="51"/>
       <c r="E6" s="51"/>
@@ -2046,7 +2043,7 @@
       </c>
       <c r="B8" s="51"/>
       <c r="C8" s="51" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D8" s="51"/>
       <c r="E8" s="51"/>
@@ -2072,7 +2069,7 @@
       </c>
       <c r="B9" s="51"/>
       <c r="C9" s="122" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D9" s="51"/>
       <c r="E9" s="51"/>
@@ -2100,15 +2097,15 @@
       <c r="C10" s="106" t="s">
         <v>52</v>
       </c>
-      <c r="D10" s="159" t="s">
+      <c r="D10" s="131" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="159"/>
-      <c r="F10" s="159"/>
-      <c r="G10" s="160" t="s">
+      <c r="E10" s="131"/>
+      <c r="F10" s="131"/>
+      <c r="G10" s="132" t="s">
         <v>53</v>
       </c>
-      <c r="H10" s="160"/>
+      <c r="H10" s="132"/>
       <c r="I10" s="96"/>
       <c r="J10" s="96"/>
       <c r="K10" s="96"/>
@@ -2122,7 +2119,7 @@
       <c r="S10" s="96"/>
       <c r="T10" s="96"/>
     </row>
-    <row r="11" spans="1:20" ht="113.4" customHeight="1">
+    <row r="11" spans="1:20" ht="113.45" customHeight="1">
       <c r="A11" s="44" t="s">
         <v>3</v>
       </c>
@@ -2187,19 +2184,19 @@
         <v>1</v>
       </c>
       <c r="B12" s="94" t="s">
+        <v>57</v>
+      </c>
+      <c r="C12" s="20" t="s">
         <v>58</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="D12" s="21" t="s">
         <v>59</v>
       </c>
-      <c r="D12" s="21" t="s">
+      <c r="E12" s="107" t="s">
         <v>60</v>
       </c>
-      <c r="E12" s="107" t="s">
+      <c r="F12" s="22" t="s">
         <v>61</v>
-      </c>
-      <c r="F12" s="22" t="s">
-        <v>62</v>
       </c>
       <c r="G12" s="23">
         <v>0.08</v>
@@ -2210,11 +2207,11 @@
       </c>
       <c r="I12" s="24"/>
       <c r="J12" s="91" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K12" s="22"/>
       <c r="L12" s="22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="M12" s="107">
         <v>5</v>
@@ -2229,27 +2226,25 @@
       <c r="P12" s="92"/>
       <c r="Q12" s="82"/>
       <c r="R12" s="83" t="s">
-        <v>64</v>
-      </c>
-      <c r="S12" s="123" t="s">
-        <v>54</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="S12" s="123"/>
       <c r="T12" s="76" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="13" spans="1:20" s="1" customFormat="1" ht="56.4" customHeight="1">
+    <row r="13" spans="1:20" s="1" customFormat="1" ht="56.45" customHeight="1">
       <c r="A13" s="52"/>
-      <c r="B13" s="146" t="s">
+      <c r="B13" s="137" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="146"/>
-      <c r="D13" s="146"/>
-      <c r="E13" s="150">
+      <c r="C13" s="137"/>
+      <c r="D13" s="137"/>
+      <c r="E13" s="141">
         <f>SUMPRODUCT(E12:E12,F12:F12)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="150"/>
+      <c r="F13" s="141"/>
       <c r="G13" s="73">
         <f>SUMPRODUCT(E12:E12,F12:F12,G12:G12)</f>
         <v>0</v>
@@ -2259,15 +2254,15 @@
         <v>#VALUE!</v>
       </c>
       <c r="I13" s="54"/>
-      <c r="J13" s="146" t="s">
+      <c r="J13" s="137" t="s">
         <v>24</v>
       </c>
-      <c r="K13" s="146"/>
-      <c r="L13" s="150">
+      <c r="K13" s="137"/>
+      <c r="L13" s="141">
         <f>SUMPRODUCT(L12:L12,M12:M12)</f>
         <v>0</v>
       </c>
-      <c r="M13" s="150"/>
+      <c r="M13" s="141"/>
       <c r="N13" s="73">
         <f>SUMPRODUCT(L12:L12,M12:M12,N12:N12)</f>
         <v>0</v>
@@ -2294,13 +2289,13 @@
     <row r="14" spans="1:20" ht="46.5" customHeight="1">
       <c r="A14" s="56"/>
       <c r="B14" s="56"/>
-      <c r="C14" s="151"/>
-      <c r="D14" s="152"/>
-      <c r="E14" s="125" t="e">
+      <c r="C14" s="142"/>
+      <c r="D14" s="143"/>
+      <c r="E14" s="147" t="e">
         <f>SUMIF(N12:N12,"0",H12:H12)</f>
         <v>#VALUE!</v>
       </c>
-      <c r="F14" s="125"/>
+      <c r="F14" s="147"/>
       <c r="G14" s="101" t="s">
         <v>28</v>
       </c>
@@ -2309,15 +2304,15 @@
         <v>#VALUE!</v>
       </c>
       <c r="I14" s="104"/>
-      <c r="J14" s="126" t="s">
+      <c r="J14" s="148" t="s">
         <v>34</v>
       </c>
-      <c r="K14" s="126"/>
-      <c r="L14" s="126"/>
-      <c r="M14" s="127" t="s">
+      <c r="K14" s="148"/>
+      <c r="L14" s="148"/>
+      <c r="M14" s="128" t="s">
         <v>30</v>
       </c>
-      <c r="N14" s="128"/>
+      <c r="N14" s="129"/>
       <c r="O14" s="117" t="e">
         <f>O13+Q13</f>
         <v>#VALUE!</v>
@@ -2325,10 +2320,10 @@
       <c r="P14" s="116" t="s">
         <v>22</v>
       </c>
-      <c r="Q14" s="132" t="s">
+      <c r="Q14" s="151" t="s">
         <v>39</v>
       </c>
-      <c r="R14" s="133"/>
+      <c r="R14" s="152"/>
       <c r="S14" s="115"/>
       <c r="T14" s="116" t="s">
         <v>22</v>
@@ -2344,21 +2339,21 @@
       <c r="G15" s="57"/>
       <c r="H15" s="59"/>
       <c r="I15" s="104"/>
-      <c r="J15" s="126"/>
-      <c r="K15" s="126"/>
-      <c r="L15" s="126"/>
-      <c r="M15" s="129" t="s">
+      <c r="J15" s="148"/>
+      <c r="K15" s="148"/>
+      <c r="L15" s="148"/>
+      <c r="M15" s="130" t="s">
         <v>37</v>
       </c>
-      <c r="N15" s="129"/>
+      <c r="N15" s="130"/>
       <c r="O15" s="99"/>
       <c r="P15" s="100" t="s">
         <v>22</v>
       </c>
-      <c r="Q15" s="130" t="s">
+      <c r="Q15" s="149" t="s">
         <v>43</v>
       </c>
-      <c r="R15" s="131"/>
+      <c r="R15" s="150"/>
       <c r="S15" s="108"/>
       <c r="T15" s="100" t="s">
         <v>22</v>
@@ -2374,23 +2369,23 @@
       <c r="G16" s="58"/>
       <c r="H16" s="59"/>
       <c r="I16" s="104"/>
-      <c r="J16" s="158" t="s">
+      <c r="J16" s="127" t="s">
         <v>35</v>
       </c>
-      <c r="K16" s="158"/>
-      <c r="L16" s="158"/>
-      <c r="M16" s="127" t="s">
+      <c r="K16" s="127"/>
+      <c r="L16" s="127"/>
+      <c r="M16" s="128" t="s">
         <v>30</v>
       </c>
-      <c r="N16" s="128"/>
+      <c r="N16" s="129"/>
       <c r="O16" s="117"/>
       <c r="P16" s="116" t="s">
         <v>22</v>
       </c>
-      <c r="Q16" s="132" t="s">
+      <c r="Q16" s="151" t="s">
         <v>39</v>
       </c>
-      <c r="R16" s="133"/>
+      <c r="R16" s="152"/>
       <c r="S16" s="115"/>
       <c r="T16" s="116" t="s">
         <v>22</v>
@@ -2406,21 +2401,21 @@
       <c r="G17" s="58"/>
       <c r="H17" s="59"/>
       <c r="I17" s="104"/>
-      <c r="J17" s="158"/>
-      <c r="K17" s="158"/>
-      <c r="L17" s="158"/>
-      <c r="M17" s="129" t="s">
+      <c r="J17" s="127"/>
+      <c r="K17" s="127"/>
+      <c r="L17" s="127"/>
+      <c r="M17" s="130" t="s">
         <v>37</v>
       </c>
-      <c r="N17" s="129"/>
+      <c r="N17" s="130"/>
       <c r="O17" s="99"/>
       <c r="P17" s="100" t="s">
         <v>22</v>
       </c>
-      <c r="Q17" s="130" t="s">
+      <c r="Q17" s="149" t="s">
         <v>43</v>
       </c>
-      <c r="R17" s="131"/>
+      <c r="R17" s="150"/>
       <c r="S17" s="108"/>
       <c r="T17" s="100" t="s">
         <v>22</v>
@@ -2428,11 +2423,11 @@
     </row>
     <row r="18" spans="1:22" ht="41.25" customHeight="1">
       <c r="B18" s="62"/>
-      <c r="C18" s="141" t="s">
+      <c r="C18" s="160" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="141"/>
-      <c r="E18" s="142"/>
+      <c r="D18" s="160"/>
+      <c r="E18" s="161"/>
       <c r="F18" s="121">
         <v>270000</v>
       </c>
@@ -2440,7 +2435,7 @@
         <v>22</v>
       </c>
       <c r="H18" s="63" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="I18" s="63"/>
       <c r="J18" s="109"/>
@@ -2459,11 +2454,11 @@
     </row>
     <row r="19" spans="1:22" ht="41.25" customHeight="1">
       <c r="B19" s="62"/>
-      <c r="C19" s="139" t="s">
+      <c r="C19" s="158" t="s">
         <v>45</v>
       </c>
-      <c r="D19" s="139"/>
-      <c r="E19" s="140"/>
+      <c r="D19" s="158"/>
+      <c r="E19" s="159"/>
       <c r="F19" s="121" t="e">
         <f>#REF!</f>
         <v>#REF!</v>
@@ -2489,11 +2484,11 @@
     </row>
     <row r="20" spans="1:22" ht="41.25" customHeight="1">
       <c r="B20" s="62"/>
-      <c r="C20" s="137" t="s">
+      <c r="C20" s="156" t="s">
         <v>44</v>
       </c>
-      <c r="D20" s="137"/>
-      <c r="E20" s="138"/>
+      <c r="D20" s="156"/>
+      <c r="E20" s="157"/>
       <c r="F20" s="61" t="e">
         <f>S13-F18-F19</f>
         <v>#VALUE!</v>
@@ -2509,8 +2504,8 @@
       <c r="M20" s="112"/>
       <c r="N20" s="60"/>
       <c r="O20" s="118"/>
-      <c r="P20" s="136"/>
-      <c r="Q20" s="136"/>
+      <c r="P20" s="155"/>
+      <c r="Q20" s="155"/>
       <c r="R20" s="119"/>
       <c r="S20" s="119"/>
       <c r="T20" s="119"/>
@@ -2542,36 +2537,36 @@
       <c r="V21" s="66"/>
     </row>
     <row r="22" spans="1:22" ht="51" customHeight="1">
-      <c r="A22" s="144" t="s">
+      <c r="A22" s="135" t="s">
         <v>38</v>
       </c>
-      <c r="B22" s="144"/>
-      <c r="C22" s="144"/>
-      <c r="D22" s="144" t="s">
+      <c r="B22" s="135"/>
+      <c r="C22" s="135"/>
+      <c r="D22" s="135" t="s">
         <v>6</v>
       </c>
-      <c r="E22" s="144"/>
-      <c r="F22" s="144"/>
-      <c r="G22" s="149" t="s">
+      <c r="E22" s="135"/>
+      <c r="F22" s="135"/>
+      <c r="G22" s="140" t="s">
         <v>7</v>
       </c>
-      <c r="H22" s="149"/>
+      <c r="H22" s="140"/>
       <c r="I22" s="67"/>
-      <c r="J22" s="144" t="s">
+      <c r="J22" s="135" t="s">
         <v>8</v>
       </c>
-      <c r="K22" s="144"/>
-      <c r="L22" s="144"/>
-      <c r="M22" s="144"/>
-      <c r="N22" s="144"/>
+      <c r="K22" s="135"/>
+      <c r="L22" s="135"/>
+      <c r="M22" s="135"/>
+      <c r="N22" s="135"/>
       <c r="O22" s="63"/>
       <c r="P22" s="71"/>
       <c r="Q22" s="84"/>
-      <c r="R22" s="124" t="s">
+      <c r="R22" s="146" t="s">
         <v>49</v>
       </c>
-      <c r="S22" s="124"/>
-      <c r="T22" s="124"/>
+      <c r="S22" s="146"/>
+      <c r="T22" s="146"/>
     </row>
     <row r="23" spans="1:22" ht="48.75" customHeight="1">
       <c r="A23" s="60"/>
@@ -2591,11 +2586,11 @@
       <c r="O23" s="64"/>
       <c r="P23" s="60"/>
       <c r="Q23" s="85"/>
-      <c r="R23" s="124"/>
-      <c r="S23" s="124"/>
-      <c r="T23" s="124"/>
-    </row>
-    <row r="24" spans="1:22" ht="58.2" customHeight="1">
+      <c r="R23" s="146"/>
+      <c r="S23" s="146"/>
+      <c r="T23" s="146"/>
+    </row>
+    <row r="24" spans="1:22" ht="58.15" customHeight="1">
       <c r="A24" s="60"/>
       <c r="B24" s="60"/>
       <c r="C24" s="64"/>
@@ -2613,9 +2608,9 @@
       <c r="O24" s="64"/>
       <c r="P24" s="60"/>
       <c r="Q24" s="85"/>
-      <c r="R24" s="124"/>
-      <c r="S24" s="124"/>
-      <c r="T24" s="124"/>
+      <c r="R24" s="146"/>
+      <c r="S24" s="146"/>
+      <c r="T24" s="146"/>
     </row>
     <row r="25" spans="1:22" ht="48.75" customHeight="1">
       <c r="A25" s="60"/>
@@ -2635,52 +2630,52 @@
       <c r="O25" s="64"/>
       <c r="P25" s="60"/>
       <c r="Q25" s="85"/>
-      <c r="R25" s="124"/>
-      <c r="S25" s="124"/>
-      <c r="T25" s="124"/>
+      <c r="R25" s="146"/>
+      <c r="S25" s="146"/>
+      <c r="T25" s="146"/>
     </row>
     <row r="26" spans="1:22" ht="51.6" customHeight="1">
-      <c r="A26" s="154" t="str">
+      <c r="A26" s="145" t="str">
         <f>+C6</f>
         <v>{User}</v>
       </c>
-      <c r="B26" s="154"/>
-      <c r="C26" s="154"/>
-      <c r="D26" s="134"/>
-      <c r="E26" s="134"/>
-      <c r="F26" s="134"/>
-      <c r="G26" s="153" t="s">
+      <c r="B26" s="145"/>
+      <c r="C26" s="145"/>
+      <c r="D26" s="153"/>
+      <c r="E26" s="153"/>
+      <c r="F26" s="153"/>
+      <c r="G26" s="144" t="s">
         <v>48</v>
       </c>
-      <c r="H26" s="153"/>
+      <c r="H26" s="144"/>
       <c r="I26" s="16"/>
-      <c r="J26" s="135"/>
-      <c r="K26" s="135"/>
-      <c r="L26" s="135"/>
-      <c r="M26" s="135"/>
-      <c r="N26" s="135"/>
+      <c r="J26" s="154"/>
+      <c r="K26" s="154"/>
+      <c r="L26" s="154"/>
+      <c r="M26" s="154"/>
+      <c r="N26" s="154"/>
       <c r="O26" s="16"/>
       <c r="P26" s="27"/>
       <c r="Q26" s="18"/>
-      <c r="R26" s="124"/>
-      <c r="S26" s="124"/>
-      <c r="T26" s="124"/>
+      <c r="R26" s="146"/>
+      <c r="S26" s="146"/>
+      <c r="T26" s="146"/>
     </row>
     <row r="27" spans="1:22" ht="114" customHeight="1">
-      <c r="A27" s="143"/>
-      <c r="B27" s="143"/>
-      <c r="C27" s="143"/>
-      <c r="D27" s="147"/>
-      <c r="E27" s="147"/>
-      <c r="F27" s="147"/>
-      <c r="G27" s="148"/>
-      <c r="H27" s="148"/>
+      <c r="A27" s="134"/>
+      <c r="B27" s="134"/>
+      <c r="C27" s="134"/>
+      <c r="D27" s="138"/>
+      <c r="E27" s="138"/>
+      <c r="F27" s="138"/>
+      <c r="G27" s="139"/>
+      <c r="H27" s="139"/>
       <c r="I27" s="29"/>
-      <c r="J27" s="147"/>
-      <c r="K27" s="147"/>
-      <c r="L27" s="147"/>
-      <c r="M27" s="147"/>
-      <c r="N27" s="147"/>
+      <c r="J27" s="138"/>
+      <c r="K27" s="138"/>
+      <c r="L27" s="138"/>
+      <c r="M27" s="138"/>
+      <c r="N27" s="138"/>
       <c r="O27" s="43"/>
       <c r="P27" s="29"/>
       <c r="Q27" s="18"/>
@@ -2908,16 +2903,21 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="G1:T1"/>
-    <mergeCell ref="A4:T4"/>
-    <mergeCell ref="G2:T2"/>
-    <mergeCell ref="G3:T3"/>
-    <mergeCell ref="J16:L17"/>
-    <mergeCell ref="M16:N16"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="D10:F10"/>
-    <mergeCell ref="G10:H10"/>
-    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="R22:T26"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="J14:L15"/>
+    <mergeCell ref="M14:N14"/>
+    <mergeCell ref="M15:N15"/>
+    <mergeCell ref="Q17:R17"/>
+    <mergeCell ref="Q16:R16"/>
+    <mergeCell ref="Q15:R15"/>
+    <mergeCell ref="Q14:R14"/>
+    <mergeCell ref="D26:F26"/>
+    <mergeCell ref="J26:N26"/>
+    <mergeCell ref="P20:Q20"/>
+    <mergeCell ref="C20:E20"/>
+    <mergeCell ref="C19:E19"/>
+    <mergeCell ref="C18:E18"/>
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="D22:F22"/>
@@ -2934,33 +2934,25 @@
     <mergeCell ref="C14:D14"/>
     <mergeCell ref="G26:H26"/>
     <mergeCell ref="A26:C26"/>
-    <mergeCell ref="R22:T26"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="J14:L15"/>
-    <mergeCell ref="M14:N14"/>
-    <mergeCell ref="M15:N15"/>
-    <mergeCell ref="Q17:R17"/>
-    <mergeCell ref="Q16:R16"/>
-    <mergeCell ref="Q15:R15"/>
-    <mergeCell ref="Q14:R14"/>
-    <mergeCell ref="D26:F26"/>
-    <mergeCell ref="J26:N26"/>
-    <mergeCell ref="P20:Q20"/>
-    <mergeCell ref="C20:E20"/>
-    <mergeCell ref="C19:E19"/>
-    <mergeCell ref="C18:E18"/>
+    <mergeCell ref="G1:T1"/>
+    <mergeCell ref="A4:T4"/>
+    <mergeCell ref="G2:T2"/>
+    <mergeCell ref="G3:T3"/>
+    <mergeCell ref="J16:L17"/>
+    <mergeCell ref="M16:N16"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="D10:F10"/>
+    <mergeCell ref="G10:H10"/>
+    <mergeCell ref="E5:G5"/>
   </mergeCells>
   <phoneticPr fontId="27" type="noConversion"/>
-  <hyperlinks>
-    <hyperlink ref="S12" r:id="rId1" display="https://shopee.vn/20-N%C3%BAt-%C4%91%E1%BB%87m-cao-su-3M-SJ5312-(N%C3%BAt-d%E1%BA%B9t)-V%C3%A0-30-N%C3%BAt-3MSJ5302-(N%C3%BAt-V%C3%B2m-Nh%E1%BB%8F)-i.50663522.7926817811?sp_atk=12653609-96c4-49c5-ad3a-5eb6b2bceb18&amp;xptdk=12653609-96c4-49c5-ad3a-5eb6b2bceb18" xr:uid="{D54FCF15-44CA-4D35-98AB-373902F611F2}"/>
-  </hyperlinks>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.27559055118110237" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.15748031496062992"/>
-  <pageSetup paperSize="9" scale="33" orientation="landscape" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="33" orientation="landscape" r:id="rId1"/>
   <headerFooter alignWithMargins="0"/>
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="35" max="16383" man="1"/>
   </rowBreaks>
-  <drawing r:id="rId3"/>
-  <legacyDrawing r:id="rId4"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>